<commit_message>
Initial commit: Lead Generation Automation Pipeline
</commit_message>
<xml_diff>
--- a/Output_Leads_Sample1.xlsx
+++ b/Output_Leads_Sample1.xlsx
@@ -1041,32 +1041,32 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MahNik Systems</t>
+          <t>Computer Squad</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>contact@mahniksystems.com</t>
+          <t>contact@computersquad.ca</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>info@mahniksystems.com | hello@mahniksystems.com | support@mahniksystems.com | sales@mahniksystems.com</t>
+          <t>info@computersquad.ca | hello@computersquad.ca | support@computersquad.ca | sales@computersquad.ca</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.mahniksystems.com/</t>
+          <t>https://www.computersquad.ca/</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>mahniksystems.com</t>
+          <t>computersquad.ca</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>177 Lindyou Rd, North York, ON M9M 2B8</t>
+          <t>17 Anndale Drive, Toronto, ON M2N 2W7</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1078,32 +1078,32 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Computer Squad</t>
+          <t>MahNik Systems</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>contact@computersquad.ca</t>
+          <t>contact@mahniksystems.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>info@computersquad.ca | hello@computersquad.ca | support@computersquad.ca | sales@computersquad.ca</t>
+          <t>info@mahniksystems.com | hello@mahniksystems.com | support@mahniksystems.com | sales@mahniksystems.com</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://www.computersquad.ca/</t>
+          <t>https://www.mahniksystems.com/</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>computersquad.ca</t>
+          <t>mahniksystems.com</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>17 Anndale Drive, Toronto, ON M2N 2W7</t>
+          <t>177 Lindyou Rd, North York, ON M9M 2B8</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">

</xml_diff>